<commit_message>
Separate English and Chinese versions of every free resource
Separate English and Chinese Excel dashboards and previews; download matches
the page language. Status options, screen-reader labels, unlock message and
sample names now switch language instead of showing both.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018jGRoRsjqrs6YVu7sosPUR
</commit_message>
<xml_diff>
--- a/files/production-kpi-dashboard.xlsx
+++ b/files/production-kpi-dashboard.xlsx
@@ -71,138 +71,27 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="82">
-  <si>
-    <r>
-      <rPr>
-        <i val="true"/>
-        <sz val="10"/>
-        <color rgb="FF5B6B78"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Updates automatically from Daily Log. Do not type here.  </t>
-    </r>
-    <r>
-      <rPr>
-        <i val="true"/>
-        <sz val="10"/>
-        <color rgb="FF5B6B78"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">自动更新，请勿在此输入。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <color rgb="FFFF7A1A"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">DOWNTIME PARETO  ·  </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <color rgb="FFFF7A1A"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">停机 </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <color rgb="FFFF7A1A"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Pareto</t>
-    </r>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="74">
+  <si>
+    <t xml:space="preserve">Updates automatically from Daily Log. Do not type here.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DOWNTIME PARETO</t>
   </si>
   <si>
     <t xml:space="preserve">Helper (do not edit)</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <color rgb="FFFF7A1A"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">MONTH SUMMARY  ·  </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <color rgb="FFFF7A1A"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">月度汇总</t>
-    </r>
+    <t xml:space="preserve">MONTH SUMMARY</t>
   </si>
   <si>
     <t xml:space="preserve">#</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Reason  ·  </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">原因</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Minutes  ·  </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">分钟</t>
-    </r>
+    <t xml:space="preserve">Reason</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minutes</t>
   </si>
   <si>
     <t xml:space="preserve">% of total</t>
@@ -211,1001 +100,103 @@
     <t xml:space="preserve">Cumulative %</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Days recorded  ·  </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">记录天数</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Good units  ·  </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">良品总数</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Target  ·  </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">目标</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Attainment  ·  </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">达成率</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Availability  ·  </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">稼动率</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Performance  ·  </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">性能率</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Quality  ·  </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">良率</t>
-    </r>
+    <t xml:space="preserve">Days recorded</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Good units</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Target</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Attainment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Availability</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Performance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quality</t>
   </si>
   <si>
     <t xml:space="preserve">OEE</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">OEE target  ·  OEE </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">目标</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Scrap %  ·  </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">报废率</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <i val="true"/>
-        <sz val="10"/>
-        <color rgb="FF5B6B78"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Fix the top 1–2 reasons first; they are usually most of the loss.  </t>
-    </r>
-    <r>
-      <rPr>
-        <i val="true"/>
-        <sz val="10"/>
-        <color rgb="FF5B6B78"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">先解决前 </t>
-    </r>
-    <r>
-      <rPr>
-        <i val="true"/>
-        <sz val="10"/>
-        <color rgb="FF5B6B78"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1–2 </t>
-    </r>
-    <r>
-      <rPr>
-        <i val="true"/>
-        <sz val="10"/>
-        <color rgb="FF5B6B78"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">个原因，它们通常占大部分损失。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Downtime (hours)  ·  </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">停机（小时）</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Biggest loss  ·  </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">最大损失</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="16"/>
-        <color rgb="FF0B2B44"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Production KPI Dashboard  ·  </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="16"/>
-        <color rgb="FF0B2B44"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">生产 </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="16"/>
-        <color rgb="FF0B2B44"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">KPI </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="16"/>
-        <color rgb="FF0B2B44"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">仪表板</t>
-    </r>
+    <t xml:space="preserve">OEE target</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scrap %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fix the top 1–2 reasons first; they are usually most of the loss.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Downtime (hours)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Biggest loss</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Production KPI Dashboard</t>
   </si>
   <si>
     <t xml:space="preserve">Free template by LAOYU (@laoyu.talks)  ·  laoyutalks-max.github.io/laoyutalks-content-brain</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <color rgb="FFFF7A1A"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">HOW TO USE  ·  </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <color rgb="FFFF7A1A"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">使用方法</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1. Settings: enter your line name, month start date, planned minutes per day, ideal cycle time and targets.   </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">在 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Settings </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">填写产线、月份开始日期、每天计划时间、理想节拍和目标。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2. Daily Log: each day, fill the yellow cells: downtime minutes, total units, good units, main downtime reason.   </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">每天在 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Daily Log </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">填写黄色格：停机分钟、总产量、良品数、主要停机原因。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3. Downtime Log (optional): log each stop with its reason and minutes for a more accurate Pareto.   </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">（可选）在 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Downtime Log </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">记录每次停机原因与时长，</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Pareto </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">更准确。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">4. Dashboard: everything else updates by itself. Do not type in white cells; they contain formulas.   Dashboard </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">会自动更新。白色格是公式，请不要输入。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <color rgb="FFFF7A1A"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">LEGEND  ·  </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <color rgb="FFFF7A1A"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">图例</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Yellow cell = enter your data   </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">黄色格 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">= </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">输入数据</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Blue text = sample numbers (October 2026 example). Replace them with your own.   </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">蓝色字 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">= </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">示例数据（</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">2026 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">年 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">月），请替换成你自己的。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <color rgb="FFFF7A1A"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">DEFINITIONS  ·  </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <color rgb="FFFF7A1A"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">定义</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Availability = Run time ÷ Planned time   (Run time = Planned time − Downtime)   </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">稼动率 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">= </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">运行时间 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">÷ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">计划时间</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Performance = (Ideal cycle time × Total units) ÷ Run time   </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">性能率 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">= </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">理想节拍 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">× </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">总产量 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">÷ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">运行时间</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Quality = Good units ÷ Total units   </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">良率 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">= </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">良品数 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">÷ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">总产量</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">OEE = Availability × Performance × Quality   OEE = </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">稼动率 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">× </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">性能率 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">× </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">良率</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Monthly figures are calculated from monthly totals, not by averaging daily percentages.   </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">月度数据由月度总数计算，而不是平均每日百分比。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <color rgb="FFFF7A1A"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">TIP  ·  </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <color rgb="FFFF7A1A"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">提示</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">High availability with flat output usually means speed losses or minor stops. Look at Performance, not only Availability.   </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">稼动率高但产量没变，通常是速度损失或小停机。要看性能率，而不只是稼动率。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="16"/>
-        <color rgb="FF0B2B44"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Settings  ·  </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="16"/>
-        <color rgb="FF0B2B44"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">设置</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Line / area  ·  </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">产线 </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/ </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">区域</t>
-    </r>
+    <t xml:space="preserve">HOW TO USE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Settings: enter your line name, month start date, planned minutes per day, ideal cycle time and targets.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Daily Log: each day, fill the yellow cells: downtime minutes, total units, good units and the main downtime reason.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Downtime Log (optional): log each stop with its reason and minutes for a more accurate Pareto.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Dashboard: everything else updates by itself. Do not type in white cells; they contain formulas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LEGEND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yellow cell = enter your data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blue text = sample numbers (October 2026 example). Replace them with your own.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DEFINITIONS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Availability = Run time ÷ Planned time   (Run time = Planned time − Downtime)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Performance = (Ideal cycle time × Total units) ÷ Run time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quality = Good units ÷ Total units</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OEE = Availability × Performance × Quality</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monthly figures are calculated from monthly totals, not by averaging daily percentages.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TIP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High availability with flat output usually means speed losses or minor stops. Look at Performance, not only Availability.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Settings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Line / area</t>
   </si>
   <si>
     <t xml:space="preserve">Line A</t>
@@ -1214,116 +205,25 @@
     <t xml:space="preserve">Name shown on the dashboard</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Month start date  ·  </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">月份开始日期</t>
-    </r>
+    <t xml:space="preserve">Month start date</t>
   </si>
   <si>
     <t xml:space="preserve">First day of the month you are tracking</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Planned production time per day (min)  ·  </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">每天计划生产时间（分钟）</t>
-    </r>
+    <t xml:space="preserve">Planned production time per day (min)</t>
   </si>
   <si>
     <t xml:space="preserve">Shift time minus planned breaks. Sample: 8 h shift minus 30 min breaks</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Ideal cycle time (seconds per unit)  ·  </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">理想节拍（秒</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">件）</t>
-    </r>
+    <t xml:space="preserve">Ideal cycle time (seconds per unit)</t>
   </si>
   <si>
     <t xml:space="preserve">Fastest proven cycle time for this product (sample value)</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Daily output target (good units)  ·  </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">每日产量目标（良品）</t>
-    </r>
+    <t xml:space="preserve">Daily output target (good units)</t>
   </si>
   <si>
     <t xml:space="preserve">Sample target</t>
@@ -1332,722 +232,86 @@
     <t xml:space="preserve">Sample target. 85% is often quoted as world class; set a realistic target for your line</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Scrap target  ·  </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">报废率目标</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <color rgb="FFFF7A1A"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Downtime reasons  ·  </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <color rgb="FFFF7A1A"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">停机原因 </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <color rgb="FFFF7A1A"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(edit the list to match your line)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Breakdown · </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">故障</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Changeover · </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">换线</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Waiting material · </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">等料</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">No operator · </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">缺人</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Quality hold · </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">质量隔离</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Planned maintenance · </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">计划保养</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Minor stops · </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">小停机</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Other · </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">其他</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Date
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">日期</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Planned (min)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">计划时间</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Downtime (min)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">停机</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Total units
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">总产量</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Good units
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">良品</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Main downtime reason
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">主要停机原因</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Notes
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">备注</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Run time (min)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">运行时间</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Availability
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">稼动率</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Performance
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">性能率</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Quality
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">良率</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Target
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">目标</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">vs Target
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">达成率</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Scrap units
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">报废数</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Scrap %
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">报废率</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Reason
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">原因</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Minutes
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">分钟</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Machine / station
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">设备 </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/ </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">工位</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Note
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">备注</t>
-    </r>
+    <t xml:space="preserve">Scrap target</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Downtime reasons (edit the list to match your line)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Breakdown</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Changeover</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Waiting material</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No operator</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quality hold</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Planned maintenance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minor stops</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Other</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Planned (min)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Downtime (min)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total units</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Main downtime reason</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run time (min)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vs Target</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scrap units</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Machine / station</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Note</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="9">
+  <numFmts count="10">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0"/>
     <numFmt numFmtId="166" formatCode="#,##0"/>
     <numFmt numFmtId="167" formatCode="0%"/>
-    <numFmt numFmtId="168" formatCode="0.0%"/>
-    <numFmt numFmtId="169" formatCode="#,##0.0"/>
-    <numFmt numFmtId="170" formatCode="@"/>
-    <numFmt numFmtId="171" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="172" formatCode="ddd\ dd\-mmm"/>
+    <numFmt numFmtId="168" formatCode="General"/>
+    <numFmt numFmtId="169" formatCode="0.0%"/>
+    <numFmt numFmtId="170" formatCode="#,##0.0"/>
+    <numFmt numFmtId="171" formatCode="@"/>
+    <numFmt numFmtId="172" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="173" formatCode="ddd\ dd\-mmm"/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2087,26 +351,12 @@
       <charset val="1"/>
     </font>
     <font>
-      <i val="true"/>
-      <sz val="10"/>
-      <color rgb="FF5B6B78"/>
-      <name val="Noto Sans CJK SC"/>
-      <family val="2"/>
-    </font>
-    <font>
       <b val="true"/>
       <sz val="11"/>
       <color rgb="FFFF7A1A"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="11"/>
-      <color rgb="FFFF7A1A"/>
-      <name val="Noto Sans CJK SC"/>
-      <family val="2"/>
     </font>
     <font>
       <b val="true"/>
@@ -2119,22 +369,9 @@
     <font>
       <b val="true"/>
       <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Noto Sans CJK SC"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <name val="Noto Sans CJK SC"/>
-      <family val="2"/>
     </font>
     <font>
       <b val="true"/>
@@ -2151,24 +388,10 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="8"/>
-      <color rgb="FF999999"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
       <b val="true"/>
       <sz val="18"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="18"/>
-      <color rgb="FF000000"/>
-      <name val="Noto Sans CJK SC"/>
       <family val="2"/>
     </font>
     <font>
@@ -2178,36 +401,11 @@
       <family val="2"/>
     </font>
     <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="16"/>
-      <color rgb="FF0B2B44"/>
-      <name val="Noto Sans CJK SC"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Noto Sans CJK SC"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF0000FF"/>
-      <name val="Noto Sans CJK SC"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -2297,83 +495,83 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="171" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="22" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="172" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="22" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="22" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="173" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2381,15 +579,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="22" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2470,7 +668,7 @@
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF7A1A"/>
       <rgbColor rgb="FF5B6B78"/>
-      <rgbColor rgb="FF999999"/>
+      <rgbColor rgb="FF969696"/>
       <rgbColor rgb="FF0B2B44"/>
       <rgbColor rgb="FF199E70"/>
       <rgbColor rgb="FF003300"/>
@@ -2510,7 +708,7 @@
                 </a:solidFill>
                 <a:latin typeface="Calibri"/>
               </a:rPr>
-              <a:t>Good units vs target  ·  良品 vs 目标</a:t>
+              <a:t>Good units vs target</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -2538,8 +736,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Good units
-良品</c:v>
+                  <c:v>Good units</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2757,8 +954,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="75336792"/>
-        <c:axId val="42788564"/>
+        <c:axId val="77573220"/>
+        <c:axId val="83133173"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -2772,8 +969,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Target
-目标</c:v>
+                  <c:v>Target</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -3004,11 +1200,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="75336792"/>
-        <c:axId val="42788564"/>
+        <c:axId val="77573220"/>
+        <c:axId val="83133173"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="75336792"/>
+        <c:axId val="77573220"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3040,7 +1236,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="42788564"/>
+        <c:crossAx val="83133173"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3048,7 +1244,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="42788564"/>
+        <c:axId val="83133173"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3064,40 +1260,6 @@
             </a:ln>
           </c:spPr>
         </c:majorGridlines>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr rot="-5400000"/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
-                    <a:solidFill>
-                      <a:srgbClr val="000000"/>
-                    </a:solidFill>
-                    <a:latin typeface="Calibri"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
-                    <a:solidFill>
-                      <a:srgbClr val="000000"/>
-                    </a:solidFill>
-                    <a:latin typeface="Calibri"/>
-                  </a:rPr>
-                  <a:t>Units</a:t>
-                </a:r>
-              </a:p>
-            </c:rich>
-          </c:tx>
-          <c:overlay val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln w="0">
-              <a:noFill/>
-            </a:ln>
-          </c:spPr>
-        </c:title>
         <c:numFmt formatCode="#,##0" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -3124,7 +1286,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="75336792"/>
+        <c:crossAx val="77573220"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3202,7 +1364,7 @@
                 </a:solidFill>
                 <a:latin typeface="Calibri"/>
               </a:rPr>
-              <a:t>Daily OEE  ·  每日 OEE</a:t>
+              <a:t>Daily OEE</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -3448,11 +1610,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="48037287"/>
-        <c:axId val="63370246"/>
+        <c:axId val="95811293"/>
+        <c:axId val="54835412"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="48037287"/>
+        <c:axId val="95811293"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3484,7 +1646,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="63370246"/>
+        <c:crossAx val="54835412"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3492,7 +1654,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="63370246"/>
+        <c:axId val="54835412"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="1"/>
@@ -3536,7 +1698,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="48037287"/>
+        <c:crossAx val="95811293"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3590,7 +1752,7 @@
                 </a:solidFill>
                 <a:latin typeface="Calibri"/>
               </a:rPr>
-              <a:t>Downtime by reason (min)  ·  停机原因</a:t>
+              <a:t>Downtime by reason (min)</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -3618,7 +1780,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Minutes  ·  分钟</c:v>
+                  <c:v>Minutes</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -3663,19 +1825,19 @@
               <c:strCache>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>Breakdown · 故障</c:v>
+                  <c:v>Breakdown</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Waiting material · 等料</c:v>
+                  <c:v>Waiting material</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Changeover · 换线</c:v>
+                  <c:v>Changeover</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Minor stops · 小停机</c:v>
+                  <c:v>Minor stops</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>No operator · 缺人</c:v>
+                  <c:v>No operator</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>-</c:v>
@@ -3725,11 +1887,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="95035570"/>
-        <c:axId val="40663748"/>
+        <c:axId val="9300929"/>
+        <c:axId val="16911067"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="95035570"/>
+        <c:axId val="9300929"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -3761,7 +1923,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="40663748"/>
+        <c:crossAx val="16911067"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3769,7 +1931,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="40663748"/>
+        <c:axId val="16911067"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3811,7 +1973,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="95035570"/>
+        <c:crossAx val="9300929"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3846,13 +2008,13 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>17</xdr:row>
-      <xdr:rowOff>20160</xdr:rowOff>
+      <xdr:rowOff>130680</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>200160</xdr:colOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>552600</xdr:colOff>
       <xdr:row>31</xdr:row>
-      <xdr:rowOff>52920</xdr:rowOff>
+      <xdr:rowOff>163440</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3876,13 +2038,13 @@
       <xdr:col>5</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>17</xdr:row>
-      <xdr:rowOff>20160</xdr:rowOff>
+      <xdr:rowOff>130680</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>35280</xdr:colOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>128520</xdr:colOff>
       <xdr:row>31</xdr:row>
-      <xdr:rowOff>52920</xdr:rowOff>
+      <xdr:rowOff>163440</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -3890,7 +2052,7 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="4793040" y="3429000"/>
+        <a:off x="3947040" y="3429000"/>
         <a:ext cx="5039640" cy="2699640"/>
       </xdr:xfrm>
       <a:graphic>
@@ -3906,13 +2068,13 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>33</xdr:row>
-      <xdr:rowOff>20520</xdr:rowOff>
+      <xdr:rowOff>131040</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>200160</xdr:colOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>552600</xdr:colOff>
       <xdr:row>47</xdr:row>
-      <xdr:rowOff>52920</xdr:rowOff>
+      <xdr:rowOff>163440</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -4118,12 +2280,12 @@
   <dimension ref="A1:L16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="3"/>
@@ -4142,7 +2304,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E3" s="3" t="s">
         <v>1</v>
       </c>
@@ -4150,7 +2312,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
@@ -4183,7 +2345,7 @@
       </c>
       <c r="F5" s="7" t="str">
         <f aca="false">IF(G5=0,"-",INDEX($K$5:$K$12,MATCH(LARGE($L$5:$L$12,E5),$L$5:$L$12,0)))</f>
-        <v>Breakdown · 故障</v>
+        <v>Breakdown</v>
       </c>
       <c r="G5" s="8" t="n">
         <f aca="false">ROUND(LARGE($L$5:$L$12,E5),0)</f>
@@ -4197,9 +2359,9 @@
         <f aca="false">SUM($H$5:H5)</f>
         <v>0.4</v>
       </c>
-      <c r="K5" s="10" t="str">
+      <c r="K5" s="0" t="str">
         <f aca="false">Settings!A13</f>
-        <v>Breakdown · 故障</v>
+        <v>Breakdown</v>
       </c>
       <c r="L5" s="10" t="n">
         <f aca="false">IF(COUNT('Downtime Log'!C2:C301)&gt;0,SUMIFS('Downtime Log'!C2:C301,'Downtime Log'!B2:B301,K5),SUMIFS('Daily Log'!C2:C32,'Daily Log'!F2:F32,K5))+ROW()/100000</f>
@@ -4219,7 +2381,7 @@
       </c>
       <c r="F6" s="7" t="str">
         <f aca="false">IF(G6=0,"-",INDEX($K$5:$K$12,MATCH(LARGE($L$5:$L$12,E6),$L$5:$L$12,0)))</f>
-        <v>Waiting material · 等料</v>
+        <v>Waiting material</v>
       </c>
       <c r="G6" s="8" t="n">
         <f aca="false">ROUND(LARGE($L$5:$L$12,E6),0)</f>
@@ -4233,9 +2395,9 @@
         <f aca="false">SUM($H$5:H6)</f>
         <v>0.73125</v>
       </c>
-      <c r="K6" s="10" t="str">
+      <c r="K6" s="0" t="str">
         <f aca="false">Settings!A14</f>
-        <v>Changeover · 换线</v>
+        <v>Changeover</v>
       </c>
       <c r="L6" s="10" t="n">
         <f aca="false">IF(COUNT('Downtime Log'!C2:C301)&gt;0,SUMIFS('Downtime Log'!C2:C301,'Downtime Log'!B2:B301,K6),SUMIFS('Daily Log'!C2:C32,'Daily Log'!F2:F32,K6))+ROW()/100000</f>
@@ -4255,7 +2417,7 @@
       </c>
       <c r="F7" s="7" t="str">
         <f aca="false">IF(G7=0,"-",INDEX($K$5:$K$12,MATCH(LARGE($L$5:$L$12,E7),$L$5:$L$12,0)))</f>
-        <v>Changeover · 换线</v>
+        <v>Changeover</v>
       </c>
       <c r="G7" s="8" t="n">
         <f aca="false">ROUND(LARGE($L$5:$L$12,E7),0)</f>
@@ -4269,9 +2431,9 @@
         <f aca="false">SUM($H$5:H7)</f>
         <v>0.85625</v>
       </c>
-      <c r="K7" s="10" t="str">
+      <c r="K7" s="0" t="str">
         <f aca="false">Settings!A15</f>
-        <v>Waiting material · 等料</v>
+        <v>Waiting material</v>
       </c>
       <c r="L7" s="10" t="n">
         <f aca="false">IF(COUNT('Downtime Log'!C2:C301)&gt;0,SUMIFS('Downtime Log'!C2:C301,'Downtime Log'!B2:B301,K7),SUMIFS('Daily Log'!C2:C32,'Daily Log'!F2:F32,K7))+ROW()/100000</f>
@@ -4291,7 +2453,7 @@
       </c>
       <c r="F8" s="7" t="str">
         <f aca="false">IF(G8=0,"-",INDEX($K$5:$K$12,MATCH(LARGE($L$5:$L$12,E8),$L$5:$L$12,0)))</f>
-        <v>Minor stops · 小停机</v>
+        <v>Minor stops</v>
       </c>
       <c r="G8" s="8" t="n">
         <f aca="false">ROUND(LARGE($L$5:$L$12,E8),0)</f>
@@ -4305,9 +2467,9 @@
         <f aca="false">SUM($H$5:H8)</f>
         <v>0.95</v>
       </c>
-      <c r="K8" s="10" t="str">
+      <c r="K8" s="0" t="str">
         <f aca="false">Settings!A16</f>
-        <v>No operator · 缺人</v>
+        <v>No operator</v>
       </c>
       <c r="L8" s="10" t="n">
         <f aca="false">IF(COUNT('Downtime Log'!C2:C301)&gt;0,SUMIFS('Downtime Log'!C2:C301,'Downtime Log'!B2:B301,K8),SUMIFS('Daily Log'!C2:C32,'Daily Log'!F2:F32,K8))+ROW()/100000</f>
@@ -4327,7 +2489,7 @@
       </c>
       <c r="F9" s="7" t="str">
         <f aca="false">IF(G9=0,"-",INDEX($K$5:$K$12,MATCH(LARGE($L$5:$L$12,E9),$L$5:$L$12,0)))</f>
-        <v>No operator · 缺人</v>
+        <v>No operator</v>
       </c>
       <c r="G9" s="8" t="n">
         <f aca="false">ROUND(LARGE($L$5:$L$12,E9),0)</f>
@@ -4341,9 +2503,9 @@
         <f aca="false">SUM($H$5:H9)</f>
         <v>1</v>
       </c>
-      <c r="K9" s="10" t="str">
+      <c r="K9" s="0" t="str">
         <f aca="false">Settings!A17</f>
-        <v>Quality hold · 质量隔离</v>
+        <v>Quality hold</v>
       </c>
       <c r="L9" s="10" t="n">
         <f aca="false">IF(COUNT('Downtime Log'!C2:C301)&gt;0,SUMIFS('Downtime Log'!C2:C301,'Downtime Log'!B2:B301,K9),SUMIFS('Daily Log'!C2:C32,'Daily Log'!F2:F32,K9))+ROW()/100000</f>
@@ -4377,9 +2539,9 @@
         <f aca="false">SUM($H$5:H10)</f>
         <v>1</v>
       </c>
-      <c r="K10" s="10" t="str">
+      <c r="K10" s="0" t="str">
         <f aca="false">Settings!A18</f>
-        <v>Planned maintenance · 计划保养</v>
+        <v>Planned maintenance</v>
       </c>
       <c r="L10" s="10" t="n">
         <f aca="false">IF(COUNT('Downtime Log'!C2:C301)&gt;0,SUMIFS('Downtime Log'!C2:C301,'Downtime Log'!B2:B301,K10),SUMIFS('Daily Log'!C2:C32,'Daily Log'!F2:F32,K10))+ROW()/100000</f>
@@ -4413,9 +2575,9 @@
         <f aca="false">SUM($H$5:H11)</f>
         <v>1</v>
       </c>
-      <c r="K11" s="10" t="str">
+      <c r="K11" s="0" t="str">
         <f aca="false">Settings!A19</f>
-        <v>Minor stops · 小停机</v>
+        <v>Minor stops</v>
       </c>
       <c r="L11" s="10" t="n">
         <f aca="false">IF(COUNT('Downtime Log'!C2:C301)&gt;0,SUMIFS('Downtime Log'!C2:C301,'Downtime Log'!B2:B301,K11),SUMIFS('Daily Log'!C2:C32,'Daily Log'!F2:F32,K11))+ROW()/100000</f>
@@ -4449,9 +2611,9 @@
         <f aca="false">SUM($H$5:H12)</f>
         <v>1</v>
       </c>
-      <c r="K12" s="10" t="str">
+      <c r="K12" s="0" t="str">
         <f aca="false">Settings!A20</f>
-        <v>Other · 其他</v>
+        <v>Other</v>
       </c>
       <c r="L12" s="10" t="n">
         <f aca="false">IF(COUNT('Downtime Log'!C2:C301)&gt;0,SUMIFS('Downtime Log'!C2:C301,'Downtime Log'!B2:B301,K12),SUMIFS('Daily Log'!C2:C32,'Daily Log'!F2:F32,K12))+ROW()/100000</f>
@@ -4488,13 +2650,13 @@
         <v>13.3333333333333</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
         <v>21</v>
       </c>
       <c r="B16" s="15" t="str">
         <f aca="false">IFERROR(INDEX($F$5:$F$12,1),"-")</f>
-        <v>Breakdown · 故障</v>
+        <v>Breakdown</v>
       </c>
     </row>
   </sheetData>
@@ -4536,10 +2698,10 @@
   <dimension ref="A1:A22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="150"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="120"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>22</v>
       </c>
@@ -4549,7 +2711,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
         <v>24</v>
       </c>
@@ -4574,7 +2736,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
         <v>29</v>
       </c>
@@ -4589,7 +2751,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
         <v>32</v>
       </c>
@@ -4619,7 +2781,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
         <v>38</v>
       </c>
@@ -4649,12 +2811,12 @@
   <dimension ref="A1:C20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="70"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>40</v>
       </c>
@@ -4736,7 +2898,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
         <v>54</v>
       </c>
@@ -4803,8 +2965,7 @@
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="8" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="0" width="9"/>
@@ -4826,40 +2987,40 @@
         <v>66</v>
       </c>
       <c r="E1" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" s="21" t="s">
         <v>67</v>
       </c>
-      <c r="F1" s="21" t="s">
+      <c r="G1" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="G1" s="21" t="s">
+      <c r="H1" s="21" t="s">
         <v>69</v>
       </c>
-      <c r="H1" s="21" t="s">
-        <v>70</v>
-      </c>
       <c r="I1" s="21" t="s">
-        <v>71</v>
+        <v>13</v>
       </c>
       <c r="J1" s="21" t="s">
-        <v>72</v>
+        <v>14</v>
       </c>
       <c r="K1" s="21" t="s">
-        <v>73</v>
+        <v>15</v>
       </c>
       <c r="L1" s="21" t="s">
         <v>16</v>
       </c>
       <c r="M1" s="21" t="s">
-        <v>74</v>
+        <v>11</v>
       </c>
       <c r="N1" s="21" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="O1" s="21" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="P1" s="21" t="s">
-        <v>77</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6657,27 +4818,27 @@
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="40"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="26" t="s">
         <v>63</v>
       </c>
       <c r="B1" s="26" t="s">
-        <v>78</v>
+        <v>5</v>
       </c>
       <c r="C1" s="26" t="s">
-        <v>79</v>
+        <v>6</v>
       </c>
       <c r="D1" s="26" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="E1" s="26" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>